<commit_message>
Refactor ProductionTool and CircuitInspector classes
- Removed unused method `updtoolpane` from ProductionTool.
- Cleaned up commented-out code in CircuitInspector, including the removal of the `loadcat` and `runtemp` methods.
- Added new OCR text extraction methods: `extracttext`, `extractcabnum`, and `extractprojectnames` to CircuitInspector for improved project detail extraction from PDFs.
- Updated `askprojdetails` method to utilize OCR data for pre-filling cabinet ID and project name fields in the dialog.
- Enhanced user interface feedback by highlighting auto-filled fields.
- Removed deprecated methods related to punch counting and finalization processes.
</commit_message>
<xml_diff>
--- a/Emerson.xlsx
+++ b/Emerson.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\E1547548\Desktop\New folder\pages\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E0D3740-2273-4314-9BAD-B3E3999EF69A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02C58367-9667-4EEC-98A5-1A5DCB5BE0E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -960,11 +960,11 @@
     <col min="2" max="2" width="12.6640625" style="11" customWidth="1"/>
     <col min="3" max="3" width="51.88671875" style="1" customWidth="1"/>
     <col min="4" max="4" width="15.5546875" style="1" customWidth="1"/>
-    <col min="5" max="5" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.6640625" customWidth="1"/>
     <col min="6" max="6" width="27.77734375" customWidth="1"/>
-    <col min="7" max="7" width="13.77734375" customWidth="1"/>
+    <col min="7" max="7" width="16.33203125" customWidth="1"/>
     <col min="8" max="8" width="28" customWidth="1"/>
-    <col min="9" max="9" width="14" customWidth="1"/>
+    <col min="9" max="9" width="17.77734375" customWidth="1"/>
     <col min="10" max="10" width="21.21875" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>